<commit_message>
fix: prove pending batch sessions before collection
</commit_message>
<xml_diff>
--- a/PRD/QBot核心内测Casebook_会话技能专家MCP_2026-07-29.xlsx
+++ b/PRD/QBot核心内测Casebook_会话技能专家MCP_2026-07-29.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心内测Case" sheetId="1" r:id="R38444f95618a4d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计总览" sheetId="2" r:id="Rf147f282f98948f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖矩阵" sheetId="3" r:id="R39fc36af886945f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行配置" sheetId="4" r:id="R74a2886c9b744c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据与断言" sheetId="5" r:id="R95e7c820ea7244df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case审计" sheetId="6" r:id="R5885ba46fbd44705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case收敛映射" sheetId="7" r:id="Ra7dde2fbb1e2412e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心内测Case" sheetId="1" r:id="Rb83cf16fb36f47e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计总览" sheetId="2" r:id="R575f74368f55496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖矩阵" sheetId="3" r:id="R5b2a999495ab440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行配置" sheetId="4" r:id="R59042f8da08b480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据与断言" sheetId="5" r:id="R3f8fbcd4cd42484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case审计" sheetId="6" r:id="Ra8db797c5bc8452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case收敛映射" sheetId="7" r:id="R3f40e911d36c4dbe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1701,33 +1701,34 @@
         <x:v>conversation</x:v>
       </x:c>
       <x:c r="G16" s="19" t="str">
-        <x:v>20个干净会话批量派发后按 taskId 统一回收，回复和能力状态不串任务</x:v>
+        <x:v>20个干净长任务批量派发后形成可见待回复池，再按 taskId 统一回收，回复和能力状态不串任务</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
-        <x:v>创建20个独立任务 → 立即派发 → 统一回收</x:v>
+        <x:v>创建20个独立长任务 → 立即派发 → 末条派发后截取待回复池 → 统一回收</x:v>
       </x:c>
       <x:c r="I16" s="19" t="str">
         <x:v>本轮已完成全量初始化；固定发布身份与测试账号有效；当前 Case 从干净任务开始。</x:v>
       </x:c>
       <x:c r="J16" s="19" t="str">
-        <x:v>每个任务使用唯一 run/case marker 和不同业务问题；专家/Skill/MCP 均禁用。</x:v>
+        <x:v>每个任务使用唯一 run/case marker；要求生成不少于2000字且含五个固定章节的风险评估；专家/Skill/MCP 均禁用。</x:v>
       </x:c>
       <x:c r="K16" s="19" t="str">
         <x:v>1. 建立20条带唯一marker的派发清单
-2. 逐条新建任务发送后立即切换并记录taskId
-3. 统一按taskId回收并核对prompt/reply/marker归属</x:v>
+2. 逐条新建长任务，发送后立即切换并记录taskId，不等待回复
+3. 末条派发后立即读取任务列表，至少5条显示正在执行并保存截图
+4. 统一按taskId回收并核对prompt/reply/marker归属与长回复完整性</x:v>
       </x:c>
       <x:c r="L16" s="19" t="str">
-        <x:v>20条均可回收；无错配、遗漏、重复或能力残留。</x:v>
+        <x:v>末条派发后至少5条可见“正在执行”；20条均可回收；每条回复不少于2000字；无错配、遗漏、重复或能力残留。</x:v>
       </x:c>
       <x:c r="M16" s="19" t="str">
-        <x:v>dispatched=20、collected=20、taskId唯一；每条 prompt hash 与回复归属一一对应。</x:v>
+        <x:v>dispatched=20、pending&gt;=5、collected=20、taskId唯一；每条回复长度&gt;=2000且 prompt hash 与回复归属一一对应。</x:v>
       </x:c>
       <x:c r="N16" s="19" t="str">
-        <x:v>产品行为与业务预期不符记 trusted_bug；环境/权限/目录能力不足记 trusted_blocked；执行或证据缺失记 framework_issue，禁止伪造 pass。</x:v>
+        <x:v>产品行为与业务预期不符记 trusted_bug；待回复池未形成且末条任务已完成记 testcase_issue；环境/权限/目录能力不足记 trusted_blocked；执行或证据缺失记 framework_issue，禁止伪造 pass。</x:v>
       </x:c>
       <x:c r="O16" s="19" t="str">
-        <x:v>before_screenshot,action_receipt,after_screenshot,prompt,task_id,send_receipt,transcript,reply_delta,reply_completion</x:v>
+        <x:v>before_screenshot,action_receipt,after_screenshot,public_state_readback,prompt,task_id,send_receipt,transcript,reply_delta,reply_completion</x:v>
       </x:c>
       <x:c r="P16" s="19" t="str">
         <x:v>dispatch_collect</x:v>
@@ -1748,17 +1749,17 @@
         <x:v>core-beta-action-plan/v1</x:v>
       </x:c>
       <x:c r="V16" s="19" t="str">
-        <x:v>[{"number":1,"action_id":"beta-chat-008-01","declared_step":"建立20条带唯一marker的派发清单","command":"build_dispatch_ledger","expected_state":"build_dispatch_ledger_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]},{"number":2,"action_id":"beta-chat-008-02","declared_step":"逐条新建任务发送后立即切换并记录taskId","command":"dispatch_batch_without_wait","expected_state":"dispatch_batch_without_wait_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]},{"number":3,"action_id":"beta-chat-008-03","declared_step":"统一按taskId回收并核对prompt/reply/marker归属","command":"collect_batch_by_task_id","expected_state":"collect_batch_by_task_id_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]}]</x:v>
+        <x:v>[{"number":1,"action_id":"beta-chat-008-01","declared_step":"建立20条带唯一marker的派发清单","command":"build_dispatch_ledger","expected_state":"build_dispatch_ledger_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]},{"number":2,"action_id":"beta-chat-008-02","declared_step":"逐条新建长任务，发送后立即切换并记录taskId，不等待回复","command":"dispatch_batch_without_wait","expected_state":"dispatch_batch_without_wait_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]},{"number":3,"action_id":"beta-chat-008-03","declared_step":"末条派发后立即读取任务列表，至少5条显示正在执行并保存截图","command":"assert_batch_pending_pool","expected_state":"batch_pending_pool_observed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot","public_state_readback"]},{"number":4,"action_id":"beta-chat-008-04","declared_step":"统一按taskId回收并核对prompt/reply/marker归属与长回复完整性","command":"collect_batch_by_task_id","expected_state":"collect_batch_by_task_id_completed_and_read_back","evidence_roles":["before_screenshot","action_receipt","after_screenshot"]}]</x:v>
       </x:c>
       <x:c r="W16" s="19" t="str">
-        <x:v>[{"prompt":"使用由Runner注入的唯一业务问题与case marker。","oracle":"回复只属于本任务marker","must_include":["&lt;case-marker&gt;"],"must_not_include":["&lt;other-case-marker&gt;"]}]</x:v>
-      </x:c>
-      <x:c r="X16" s="19" t="str"/>
+        <x:v>[{"prompt":"使用由Runner注入的唯一业务问题与case marker；要求不少于2000字且含五个固定章节。","oracle":"回复只属于本任务marker，长度不少于2000字，五个章节完整","must_include":["&lt;case-marker&gt;","范围与假设","用户风险","数据与隐私风险","稳定性与恢复","上线建议"],"must_not_include":["&lt;other-case-marker&gt;"]}]</x:v>
+      </x:c>
+      <x:c r="X16" s="19"/>
       <x:c r="Y16" s="19" t="str">
-        <x:v>{"pass_rule":"所有动作收据、状态读回、证据角色与业务 Oracle 同时成立：dispatched=20、collected=20、taskId唯一；每条 prompt hash 与回复归属一一对应。","fail_rule":"产品行为与业务预期不符记 trusted_bug；环境/权限/目录能力不足记 trusted_blocked；执行或证据缺失记 framework_issue，禁止伪造 pass。","block_rule":"发布身份漂移、登录/权限/目录能力不足或真实能力少于抽样下限时阻塞；不得换用随机替代能力。","hard_oracles":["dispatched=20、collected=20、taskId唯一；每条 prompt hash 与回复归属一一对应。"],"text_only_capability_claim_forbidden":false}</x:v>
+        <x:v>{"pass_rule":"所有动作收据、状态读回、证据角色与业务 Oracle 同时成立：dispatched=20、末条派发后pending&gt;=5、collected=20、taskId唯一；每条回复不少于2000字且 prompt hash 与回复归属一一对应。","fail_rule":"产品行为与业务预期不符记 trusted_bug；环境/权限/目录能力不足记 trusted_blocked；执行或证据缺失记 framework_issue，禁止伪造 pass。","block_rule":"发布身份漂移、登录/权限/目录能力不足或真实能力少于抽样下限时阻塞；不得换用随机替代能力。","hard_oracles":["dispatched=20、末条派发后pending&gt;=5、collected=20、taskId唯一；每条回复不少于2000字且 prompt hash 与回复归属一一对应。"],"text_only_capability_claim_forbidden":false,"batch_min_pending_after_dispatch":5,"batch_reply_min_chars":2000}</x:v>
       </x:c>
       <x:c r="Z16" s="19" t="str">
-        <x:v>before_screenshot,action_receipt,after_screenshot,prompt,task_id,send_receipt,transcript,reply_delta,reply_completion</x:v>
+        <x:v>before_screenshot,action_receipt,after_screenshot,public_state_readback,prompt,task_id,send_receipt,transcript,reply_delta,reply_completion</x:v>
       </x:c>
       <x:c r="AA16" s="19" t="str">
         <x:v>qbot-core-evidence/v1</x:v>
@@ -1775,7 +1776,9 @@
       <x:c r="AE16" s="19" t="str">
         <x:v>旧Case重构/合并</x:v>
       </x:c>
-      <x:c r="AF16" s="19" t="str"/>
+      <x:c r="AF16" s="19" t="str">
+        <x:v>批量派发必须留下末条派发后的任务列表截图与batch-pending-pool.json；pending阈值和回复长度均可配置，未达阈值不得可信通过。</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="82" customHeight="1">
       <x:c r="A17" s="19" t="str">
@@ -5355,7 +5358,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
-        <x:v>默认20；范围1-20；共享状态/创建/安装类仍串行</x:v>
+        <x:v>默认20；范围1-20；末条派发后pending阈值默认5；共享状态/创建/安装类仍串行</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
@@ -5444,7 +5447,7 @@
     </x:row>
     <x:row r="15" ht="62" customHeight="1">
       <x:c r="A15" s="21" t="str">
-        <x:v>执行分层：Phase 0 串行全量初始化 → Phase 1 纯会话/附件/成果按最多20条派发回收 → Phase 2 串行安装10个Skill后并发深用5个 → Phase 3 串行创建3类专家后轮转三轮会话 → Phase 4 选择5个MCP后轮转两轮会话 → Phase 5 恢复与隔离。</x:v>
+        <x:v>执行分层：Phase 0 串行全量初始化 → Phase 1 纯会话/附件/成果按最多20条派发，末条派发后先证明至少5条仍在运行，再统一回收 → Phase 2 串行安装10个Skill后并发深用5个 → Phase 3 串行创建3类专家后轮转三轮会话 → Phase 4 选择5个MCP后轮转两轮会话 → Phase 5 恢复与隔离。</x:v>
       </x:c>
       <x:c r="B15" s="21"/>
       <x:c r="C15" s="21"/>
@@ -5752,22 +5755,22 @@
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="19" t="str">
-        <x:v>pipeline_batch_size</x:v>
-      </x:c>
-      <x:c r="B5" s="19" t="n">
-        <x:v>20</x:v>
+        <x:v>pipeline_batch_size / batch_min_pending_after_dispatch / batch_reply_min_chars</x:v>
+      </x:c>
+      <x:c r="B5" s="19" t="str">
+        <x:v>20 / 5 / 2000</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>1-20</x:v>
+        <x:v>1-20 / 1-pipeline_batch_size / 500-5000</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>纯会话/附件/成果</x:v>
+        <x:v>纯会话批量派发</x:v>
       </x:c>
       <x:c r="E5" s="19" t="str">
-        <x:v>taskId唯一；dispatch=collect</x:v>
+        <x:v>末条派发后首次状态快照；taskId必须属于本批次；每条回复须满足长度及固定章节</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
-        <x:v>发送后立即切换，统一按taskId回收</x:v>
+        <x:v>统一回收前至少仍有配置数量的会话显示正在执行；三项均为可配置硬门禁</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -6021,22 +6024,22 @@
         <x:v>public_state_readback</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
-        <x:v>按钮/选择/创建/安装</x:v>
+        <x:v>设置/恢复/批量会话</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>独立API/公开capabilities/DOM状态</x:v>
+        <x:v>读取产品可见值；批量场景记录末条派发后taskId、侧栏正在执行标识、pending数量、阈值、时间和截图</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
-        <x:v>与可见状态一致</x:v>
+        <x:v>产品状态与预期一致；批量场景taskId完整且pending&gt;=5，截图与JSON一致</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>framework_issue或trusted_bug</x:v>
+        <x:v>trusted_bug/testcase_issue/framework_issue</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
-        <x:v>同一截图自证</x:v>
+        <x:v>仅点击无读回；发送时曾短暂running；仅有最终回复</x:v>
       </x:c>
       <x:c r="G6" s="19" t="str">
-        <x:v>state-readback.json</x:v>
+        <x:v>before/action/after；batch-pending-pool.json；batch-dispatch-pending-pool.png</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">

</xml_diff>